<commit_message>
discarded similar text desctiption to remove
</commit_message>
<xml_diff>
--- a/data/review/projects_to_remove_after_review.xlsx
+++ b/data/review/projects_to_remove_after_review.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jojoa\OneDrive\Dokumente\OECD\RAnalysis\PRESS\data\review\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73FEEC8F-20EC-4B20-83F7-89D9454E4483}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41A4CAF1-A838-4C7F-B52B-E794CA7E5DEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="83">
   <si>
     <t>text_mining_description</t>
   </si>
@@ -615,7 +615,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A101"/>
+  <dimension ref="A1:A87"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="255.46484375" style="2" customWidth="1"/>
@@ -1009,121 +1009,51 @@
     </row>
     <row r="78" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A78" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
     </row>
     <row r="79" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A79" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
     </row>
     <row r="80" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A80" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
     </row>
     <row r="81" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A81" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
     </row>
     <row r="82" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A82" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
     </row>
     <row r="83" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A83" t="s">
-        <v>70</v>
+        <v>78</v>
       </c>
     </row>
     <row r="84" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A84" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
     </row>
     <row r="85" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A85" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
     </row>
     <row r="86" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A86" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
     </row>
     <row r="87" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A87" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="88" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A88" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="89" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A89" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="90" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A90" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="91" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A91" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="92" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A92" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="93" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A93" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="94" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A94" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="95" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A95" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="96" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A96" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="97" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A97" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="98" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A98" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="99" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A99" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="100" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A100" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="101" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A101" t="s">
         <v>82</v>
       </c>
     </row>

</xml_diff>